<commit_message>
actualizacion del modulo de seguridad
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F767E8F-7646-4439-AF17-9573B76375CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A7EB33-E624-4282-97E0-4C5132383855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
   <sheets>
     <sheet name="ASIGNACION DE RF" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIGNACION DE RF'!$A$1:$E$34</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="74">
   <si>
     <t>RF</t>
   </si>
@@ -96,12 +99,6 @@
     <t>Gestión de Usuarios</t>
   </si>
   <si>
-    <t>⬜ 0%</t>
-  </si>
-  <si>
-    <t>🟩 100%</t>
-  </si>
-  <si>
     <t>RF-007</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
     <t>Menú Principal</t>
   </si>
   <si>
-    <t>🟨 80%</t>
-  </si>
-  <si>
     <t>Gestión de Sucursales</t>
   </si>
   <si>
@@ -180,9 +174,6 @@
     <t>Dashboard Gerencial</t>
   </si>
   <si>
-    <t>🟨 30%</t>
-  </si>
-  <si>
     <t>RF-021</t>
   </si>
   <si>
@@ -262,6 +253,12 @@
   </si>
   <si>
     <t>CESAR</t>
+  </si>
+  <si>
+    <t>COMPLETO</t>
+  </si>
+  <si>
+    <t>COMENTARIO</t>
   </si>
 </sst>
 </file>
@@ -285,12 +282,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -305,9 +308,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,490 +627,420 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}">
-  <dimension ref="A2:D35"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>
       <c r="D3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="B8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
       <c r="C8" t="s">
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>26</v>
       </c>
-      <c r="C11" t="s">
-        <v>75</v>
-      </c>
-      <c r="D11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>27</v>
       </c>
-      <c r="C12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>28</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="C13" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>31</v>
       </c>
-      <c r="C14" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
         <v>32</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>33</v>
       </c>
-      <c r="C15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>34</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>35</v>
       </c>
-      <c r="C16" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>36</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>37</v>
       </c>
-      <c r="C17" t="s">
-        <v>75</v>
-      </c>
-      <c r="D17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
         <v>38</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>39</v>
       </c>
-      <c r="C18" t="s">
-        <v>75</v>
-      </c>
-      <c r="D18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
         <v>40</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>41</v>
       </c>
-      <c r="C19" t="s">
-        <v>75</v>
-      </c>
-      <c r="D19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>42</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>43</v>
       </c>
-      <c r="C20" t="s">
-        <v>75</v>
-      </c>
-      <c r="D20" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
         <v>44</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>45</v>
       </c>
-      <c r="C21" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>46</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>47</v>
       </c>
-      <c r="C22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="B23" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>49</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>50</v>
       </c>
-      <c r="C23" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="C24" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>51</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>52</v>
       </c>
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="C25" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>53</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>54</v>
       </c>
-      <c r="C25" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="C26" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>55</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>56</v>
       </c>
-      <c r="C26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="C27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>57</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>58</v>
       </c>
-      <c r="C27" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="C28" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>59</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>60</v>
       </c>
-      <c r="C28" t="s">
-        <v>75</v>
-      </c>
-      <c r="D28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="C29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>61</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>62</v>
       </c>
-      <c r="C29" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="C30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>63</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>64</v>
       </c>
-      <c r="C30" t="s">
-        <v>75</v>
-      </c>
-      <c r="D30" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="C31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>65</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>66</v>
       </c>
-      <c r="C31" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="C32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>67</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>68</v>
       </c>
-      <c r="C32" t="s">
-        <v>75</v>
-      </c>
-      <c r="D32" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="C33" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>69</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>70</v>
       </c>
-      <c r="C33" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B34" t="s">
-        <v>72</v>
-      </c>
       <c r="C34" t="s">
         <v>5</v>
       </c>
-      <c r="D34" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>73</v>
-      </c>
-      <c r="B35" t="s">
-        <v>74</v>
-      </c>
-      <c r="C35" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" t="s">
-        <v>20</v>
-      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E34" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
RF-004 implementa gestion de seguridad, auditoria y asignacion de permisos, adicionalmente se finalizan los rfs de bitacoras de inicio de sesion y movimientos
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A7EB33-E624-4282-97E0-4C5132383855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0D7FB1-24BC-4136-9F36-8DBFC1D7C2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="ASIGNACION DE RF" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIGNACION DE RF'!$A$1:$E$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIGNACION DE RF'!$A$1:$E$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
   <si>
     <t>RF</t>
   </si>
@@ -259,6 +259,18 @@
   </si>
   <si>
     <t>COMENTARIO</t>
+  </si>
+  <si>
+    <t>modulos</t>
+  </si>
+  <si>
+    <t>cargos</t>
+  </si>
+  <si>
+    <t>empleados</t>
+  </si>
+  <si>
+    <t>rolpermisos</t>
   </si>
 </sst>
 </file>
@@ -291,7 +303,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -312,7 +324,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
@@ -653,100 +665,103 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>72</v>
+      <c r="C5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -768,10 +783,10 @@
       <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -841,7 +856,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -852,7 +867,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -863,7 +878,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -874,7 +889,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -885,7 +900,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -896,29 +911,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C22" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="C22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>49</v>
       </c>
@@ -929,7 +950,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>51</v>
       </c>
@@ -940,7 +961,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -951,7 +972,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -962,7 +983,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>57</v>
       </c>
@@ -973,7 +994,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -984,7 +1005,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -995,7 +1016,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>63</v>
       </c>
@@ -1006,7 +1027,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1017,7 +1038,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -1028,7 +1049,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -1039,8 +1060,45 @@
         <v>5</v>
       </c>
     </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B35" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B37" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E34" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}"/>
+  <autoFilter ref="A1:E37" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: actualiza RF asignados y recursos graficos
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0D7FB1-24BC-4136-9F36-8DBFC1D7C2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109A37E1-CA74-4678-AFE7-DCB45AA37636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
@@ -270,7 +270,7 @@
     <t>empleados</t>
   </si>
   <si>
-    <t>rolpermisos</t>
+    <t>ya casi</t>
   </si>
 </sst>
 </file>
@@ -294,7 +294,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -304,6 +304,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -324,7 +330,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,20 +713,17 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>77</v>
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -766,14 +769,17 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
-        <v>5</v>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update assigned requirements workbook
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A7EB33-E624-4282-97E0-4C5132383855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109A37E1-CA74-4678-AFE7-DCB45AA37636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="ASIGNACION DE RF" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIGNACION DE RF'!$A$1:$E$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIGNACION DE RF'!$A$1:$E$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
   <si>
     <t>RF</t>
   </si>
@@ -259,6 +259,18 @@
   </si>
   <si>
     <t>COMENTARIO</t>
+  </si>
+  <si>
+    <t>modulos</t>
+  </si>
+  <si>
+    <t>cargos</t>
+  </si>
+  <si>
+    <t>empleados</t>
+  </si>
+  <si>
+    <t>ya casi</t>
   </si>
 </sst>
 </file>
@@ -282,12 +294,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -312,7 +330,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
@@ -653,112 +671,115 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
-        <v>5</v>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -768,10 +789,10 @@
       <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -841,7 +862,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -852,7 +873,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -863,7 +884,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -874,7 +895,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -885,7 +906,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -896,29 +917,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C22" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="C22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>49</v>
       </c>
@@ -929,7 +956,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>51</v>
       </c>
@@ -940,7 +967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -951,7 +978,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -962,7 +989,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>57</v>
       </c>
@@ -973,7 +1000,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -984,7 +1011,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -995,7 +1022,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>63</v>
       </c>
@@ -1006,7 +1033,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1017,7 +1044,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -1028,7 +1055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -1039,8 +1066,45 @@
         <v>5</v>
       </c>
     </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B35" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B37" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E34" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}"/>
+  <autoFilter ref="A1:E37" xr:uid="{343B0E47-0565-4EF3-B140-0113EB7F4812}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implementacion del RF de clientes ya funcional
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109A37E1-CA74-4678-AFE7-DCB45AA37636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7411F3B6-4140-47AB-985C-08D6416FF804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="80">
   <si>
     <t>RF</t>
   </si>
@@ -270,7 +270,13 @@
     <t>empleados</t>
   </si>
   <si>
-    <t>ya casi</t>
+    <t xml:space="preserve">COMPLETO </t>
+  </si>
+  <si>
+    <t>PENDIENTE</t>
+  </si>
+  <si>
+    <t>60% - 70% DE AVANCE</t>
   </si>
 </sst>
 </file>
@@ -650,7 +656,7 @@
   <cols>
     <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -769,16 +775,16 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="C9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>77</v>
       </c>
     </row>
@@ -862,7 +868,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -873,7 +879,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -884,7 +890,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -895,29 +901,38 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C20" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="C20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C21" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>45</v>
       </c>
@@ -931,7 +946,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
@@ -945,29 +960,35 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C24" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="C24" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C25" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -978,7 +999,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -989,7 +1010,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>57</v>
       </c>
@@ -1000,7 +1021,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -1011,7 +1032,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -1022,7 +1043,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>63</v>
       </c>
@@ -1033,7 +1054,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -1056,14 +1077,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="A34" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C34" t="s">
-        <v>5</v>
+      <c r="C34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
implementacion de parte de inventario
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7411F3B6-4140-47AB-985C-08D6416FF804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AAE9C6-F9A4-4A51-8D4E-60B61058A4D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="81">
   <si>
     <t>RF</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>60% - 70% DE AVANCE</t>
+  </si>
+  <si>
+    <t>VERIFICAR CON EL</t>
   </si>
 </sst>
 </file>
@@ -300,7 +303,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -319,6 +322,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -332,11 +341,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -825,58 +835,75 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" t="s">
-        <v>71</v>
+      <c r="C13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
-        <v>71</v>
+      <c r="C14" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C15" t="s">
-        <v>71</v>
+      <c r="C15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C16" t="s">
-        <v>71</v>
+      <c r="C16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="A17" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C17" t="s">
-        <v>71</v>
+      <c r="C17" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1022,36 +1049,50 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="A29" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C29" t="s">
-        <v>71</v>
+      <c r="C29" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C30" t="s">
-        <v>71</v>
+      <c r="C30" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="A31" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C31" t="s">
-        <v>71</v>
+      <c r="C31" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -1066,15 +1107,16 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="A33" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C33" t="s">
-        <v>5</v>
-      </c>
+      <c r="C33" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="2"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">

</xml_diff>

<commit_message>
mejoras de varios puntos pendientes, rf inventario y entrada de inventario
</commit_message>
<xml_diff>
--- a/DOCUMENTACION/RF ASIGNADOS.xlsx
+++ b/DOCUMENTACION/RF ASIGNADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yilfe\Documents\PPI2026\PPI\DOCUMENTACION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AAE9C6-F9A4-4A51-8D4E-60B61058A4D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D0988C-6D64-4F38-AA62-406E24ADAEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0D26C389-0F52-49FE-902C-95ED8804566F}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
   <si>
     <t>RF</t>
   </si>
@@ -813,26 +813,30 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C11" t="s">
-        <v>71</v>
-      </c>
+      <c r="C11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
-        <v>71</v>
-      </c>
+      <c r="C12" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
@@ -1091,9 +1095,7 @@
         <v>71</v>
       </c>
       <c r="D31" s="4"/>
-      <c r="E31" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">

</xml_diff>